<commit_message>
CBA: rebuild without overwriting column A; notes moved to their own tab
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HvXhTSq2hCmheT3mKtqmHP
</commit_message>
<xml_diff>
--- a/output/stephen/CBA_Innovative_Advisors_Updated_2026-09-24.xlsx
+++ b/output/stephen/CBA_Innovative_Advisors_Updated_2026-09-24.xlsx
@@ -7,6 +7,7 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Notes 9-24-26" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -15,11 +16,12 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="3">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="166" formatCode="$#,##0.00"/>
   </numFmts>
-  <fonts count="9">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -69,17 +71,10 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <name val="Calibri"/>
       <b val="1"/>
-      <sz val="11"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +100,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00FFC7CE"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -165,7 +165,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="25">
+  <cellXfs count="26">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -231,21 +231,21 @@
       <alignment horizontal="center"/>
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="166" fontId="4" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
+      <protection locked="0" hidden="0"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="6" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="4" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
       <alignment horizontal="left"/>
       <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="164" fontId="7" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
-      <protection locked="0" hidden="0"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
       <protection locked="0" hidden="0"/>
     </xf>
   </cellXfs>
@@ -607,8 +607,8 @@
     <col width="15" customWidth="1" min="15" max="16"/>
     <col width="18" bestFit="1" customWidth="1" min="17" max="17"/>
     <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="30" customWidth="1" min="19" max="19"/>
-    <col width="85" customWidth="1" min="20" max="20"/>
+    <col width="32" customWidth="1" min="19" max="19"/>
+    <col width="88" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="2" ht="74.45" customHeight="1">
@@ -777,11 +777,11 @@
       <c r="P3" s="17" t="n">
         <v>200</v>
       </c>
-      <c r="Q3" s="5">
+      <c r="Q3" s="18">
         <f>M3+IF(ISNUMBER(O3),O3,0)+IF(ISNUMBER(P3),P3,0)</f>
         <v/>
       </c>
-      <c r="R3" s="18" t="inlineStr">
+      <c r="R3" s="19" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
@@ -791,9 +791,9 @@
           <t>Paychex inv 7/29/26</t>
         </is>
       </c>
-      <c r="T3" s="19" t="inlineStr">
-        <is>
-          <t>Flex Select 137.85 + Delivery 19.50 - discount 27.57 = 129.78. Matches sheet.</t>
+      <c r="T3" s="20" t="inlineStr">
+        <is>
+          <t>Flex Select 137.85 + Delivery 19.50 less discount 27.57 = 129.78. Matches the original.</t>
         </is>
       </c>
     </row>
@@ -861,23 +861,23 @@
       <c r="P4" s="17" t="n">
         <v>200</v>
       </c>
-      <c r="Q4" s="5">
+      <c r="Q4" s="18">
         <f>M4+IF(ISNUMBER(O4),O4,0)+IF(ISNUMBER(P4),P4,0)</f>
         <v/>
       </c>
-      <c r="R4" s="20" t="inlineStr">
+      <c r="R4" s="21" t="inlineStr">
         <is>
           <t>Not verified</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
         <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="T4" s="19" t="inlineStr">
-        <is>
-          <t>No invoice yet. Sheet figure retained. No 401(k) — the $0.91 was not a plan.</t>
+          <t>Eli 9/24/26</t>
+        </is>
+      </c>
+      <c r="T4" s="20" t="inlineStr">
+        <is>
+          <t>No payroll invoice yet, fee left as-is. 401(k) changed from 0.91 to 0 — that charge was not a plan.</t>
         </is>
       </c>
     </row>
@@ -945,11 +945,11 @@
       <c r="P5" s="17" t="n">
         <v>100</v>
       </c>
-      <c r="Q5" s="5">
+      <c r="Q5" s="18">
         <f>M5+IF(ISNUMBER(O5),O5,0)+IF(ISNUMBER(P5),P5,0)</f>
         <v/>
       </c>
-      <c r="R5" s="21" t="inlineStr">
+      <c r="R5" s="22" t="inlineStr">
         <is>
           <t>Corrected</t>
         </is>
@@ -959,9 +959,9 @@
           <t>Paychex inv 7/30/26</t>
         </is>
       </c>
-      <c r="T5" s="19" t="inlineStr">
-        <is>
-          <t>Sheet missed Direct Deposit Premium Processing $75.00, charged every run. 79.10 + 75.00 = 154.10.</t>
+      <c r="T5" s="20" t="inlineStr">
+        <is>
+          <t>Original missed Direct Deposit Premium Processing 75.00, charged every run. 79.10 + 75.00 = 154.10.</t>
         </is>
       </c>
     </row>
@@ -1029,11 +1029,11 @@
       <c r="P6" s="17" t="n">
         <v>200</v>
       </c>
-      <c r="Q6" s="5">
+      <c r="Q6" s="18">
         <f>M6+IF(ISNUMBER(O6),O6,0)+IF(ISNUMBER(P6),P6,0)</f>
         <v/>
       </c>
-      <c r="R6" s="20" t="inlineStr">
+      <c r="R6" s="21" t="inlineStr">
         <is>
           <t>Not verified</t>
         </is>
@@ -1043,9 +1043,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="T6" s="19" t="inlineStr">
-        <is>
-          <t>No invoice yet. Sheet figure retained.</t>
+      <c r="T6" s="20" t="inlineStr">
+        <is>
+          <t>No invoice yet. Original figure retained.</t>
         </is>
       </c>
     </row>
@@ -1117,23 +1117,23 @@
       <c r="P7" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="Q7" s="5">
+      <c r="Q7" s="18">
         <f>M7+IF(ISNUMBER(O7),O7,0)+IF(ISNUMBER(P7),P7,0)</f>
         <v/>
       </c>
-      <c r="R7" s="21" t="inlineStr">
+      <c r="R7" s="22" t="inlineStr">
         <is>
           <t>Corrected</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
         <is>
-          <t>Paychex inv 5/27/26 + HRS stmts 8/4, 9/1</t>
-        </is>
-      </c>
-      <c r="T7" s="19" t="inlineStr">
-        <is>
-          <t>Base is Officer Only Payroll 65.00, not 58.00, plus Delivery 36.00. 401(k) is 181.00/mo = 2,172.00/yr, plus 3,887.91 setup balance outstanding.</t>
+          <t>Paychex inv 5/27/26; HRS stmts 8/4, 9/1</t>
+        </is>
+      </c>
+      <c r="T7" s="20" t="inlineStr">
+        <is>
+          <t>Base is Officer Only Payroll 65.00, not 58.00, plus Delivery 36.00. 401(k) recurring 181.00/mo = 2,172.00/yr.</t>
         </is>
       </c>
     </row>
@@ -1201,11 +1201,11 @@
       <c r="P8" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="Q8" s="5">
+      <c r="Q8" s="18">
         <f>M8+IF(ISNUMBER(O8),O8,0)+IF(ISNUMBER(P8),P8,0)</f>
         <v/>
       </c>
-      <c r="R8" s="20" t="inlineStr">
+      <c r="R8" s="21" t="inlineStr">
         <is>
           <t>Not verified</t>
         </is>
@@ -1215,9 +1215,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="T8" s="19" t="inlineStr">
-        <is>
-          <t>No invoice yet. Paychex cannot link Partner Pro to this client. Prior ADP client over a year ago.</t>
+      <c r="T8" s="20" t="inlineStr">
+        <is>
+          <t>No invoice yet. Paychex cannot link Partner Pro to this client.</t>
         </is>
       </c>
     </row>
@@ -1285,11 +1285,11 @@
       <c r="P9" s="17" t="n">
         <v>0</v>
       </c>
-      <c r="Q9" s="5">
+      <c r="Q9" s="18">
         <f>M9+IF(ISNUMBER(O9),O9,0)+IF(ISNUMBER(P9),P9,0)</f>
         <v/>
       </c>
-      <c r="R9" s="18" t="inlineStr">
+      <c r="R9" s="19" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
@@ -1299,7 +1299,7 @@
           <t>Paychex inv 8/12, 8/26, 9/11/26</t>
         </is>
       </c>
-      <c r="T9" s="19" t="inlineStr">
+      <c r="T9" s="20" t="inlineStr">
         <is>
           <t>Flex Select 95.50 + Taxpay Locals 3.00 = 98.50 on all three. Semi-monthly confirmed by check dates 8/14, 8/31, 9/15.</t>
         </is>
@@ -1373,23 +1373,23 @@
       <c r="P10" s="17" t="n">
         <v>200</v>
       </c>
-      <c r="Q10" s="5">
+      <c r="Q10" s="18">
         <f>M10+IF(ISNUMBER(O10),O10,0)+IF(ISNUMBER(P10),P10,0)</f>
         <v/>
       </c>
-      <c r="R10" s="21" t="inlineStr">
+      <c r="R10" s="22" t="inlineStr">
         <is>
           <t>Corrected</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
         <is>
-          <t>Paychex inv 9/2 + 9/14/26, HRS stmts 7/5, 8/5, 9/1</t>
-        </is>
-      </c>
-      <c r="T10" s="19" t="inlineStr">
-        <is>
-          <t>Frequency, rate and headcount all corrected. HR Pro 896.70 less 394.55 discount = 502.15, bi-weekly. Invoice shows 3 active employees, not 5. 401(k) 193.00/mo = 2,316.00/yr, plus 2,749.07 setup balance outstanding.</t>
+          <t>Paychex inv 9/2 + 9/14/26; HRS stmts 7/5, 8/5, 9/1</t>
+        </is>
+      </c>
+      <c r="T10" s="20" t="inlineStr">
+        <is>
+          <t>HR Pro is a bundled HR and payroll fee, 896.70 less 394.55 discount = 502.15 per run, bi-weekly. Invoice shows 3 active employees, not 5. 401(k) recurring 193.00/mo = 2,316.00/yr.</t>
         </is>
       </c>
     </row>
@@ -1461,23 +1461,23 @@
       <c r="P11" s="17" t="n">
         <v>100</v>
       </c>
-      <c r="Q11" s="5">
+      <c r="Q11" s="18">
         <f>M11+IF(ISNUMBER(O11),O11,0)+IF(ISNUMBER(P11),P11,0)</f>
         <v/>
       </c>
-      <c r="R11" s="18" t="inlineStr">
+      <c r="R11" s="19" t="inlineStr">
         <is>
           <t>Verified</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
         <is>
-          <t>Paychex inv 8/27/26 + HRS stmts 8/4, 9/1</t>
-        </is>
-      </c>
-      <c r="T11" s="19" t="inlineStr">
-        <is>
-          <t>Express Payroll 77.00 matches sheet. 401(k) 175.00/mo = 2,100.00/yr, plus the full 3,999.00 setup balance outstanding, nothing collected yet.</t>
+          <t>Paychex inv 8/27/26; HRS stmts 8/4, 9/1</t>
+        </is>
+      </c>
+      <c r="T11" s="20" t="inlineStr">
+        <is>
+          <t>Express Payroll 77.00 matches the original. 401(k) recurring 175.00/mo = 2,100.00/yr.</t>
         </is>
       </c>
     </row>
@@ -1545,11 +1545,11 @@
       <c r="P12" s="17" t="n">
         <v>100</v>
       </c>
-      <c r="Q12" s="5">
+      <c r="Q12" s="18">
         <f>M12+IF(ISNUMBER(O12),O12,0)+IF(ISNUMBER(P12),P12,0)</f>
         <v/>
       </c>
-      <c r="R12" s="20" t="inlineStr">
+      <c r="R12" s="21" t="inlineStr">
         <is>
           <t>Not verified</t>
         </is>
@@ -1559,7 +1559,7 @@
           <t>—</t>
         </is>
       </c>
-      <c r="T12" s="19" t="inlineStr">
+      <c r="T12" s="20" t="inlineStr">
         <is>
           <t>No invoice yet. Waiting on the client to grant Partner Pro access.</t>
         </is>
@@ -1629,11 +1629,11 @@
       </c>
       <c r="O13" s="4" t="n"/>
       <c r="P13" s="4" t="n"/>
-      <c r="Q13" s="5">
+      <c r="Q13" s="18">
         <f>M13+IF(ISNUMBER(O13),O13,0)+IF(ISNUMBER(P13),P13,0)</f>
         <v/>
       </c>
-      <c r="R13" t="inlineStr">
+      <c r="R13" s="23" t="inlineStr">
         <is>
           <t>No current cost</t>
         </is>
@@ -1643,9 +1643,9 @@
           <t>Stephen 9/22/26</t>
         </is>
       </c>
-      <c r="T13" s="19" t="inlineStr">
-        <is>
-          <t>Set up at Paychex but has never run a payroll. Moving straight to ADP.</t>
+      <c r="T13" s="20" t="inlineStr">
+        <is>
+          <t>Set up at Paychex but has never run a payroll, so there is no current billing.</t>
         </is>
       </c>
     </row>
@@ -1713,11 +1713,11 @@
       </c>
       <c r="O14" s="4" t="n"/>
       <c r="P14" s="4" t="n"/>
-      <c r="Q14" s="5">
+      <c r="Q14" s="18">
         <f>M14+IF(ISNUMBER(O14),O14,0)+IF(ISNUMBER(P14),P14,0)</f>
         <v/>
       </c>
-      <c r="R14" t="inlineStr">
+      <c r="R14" s="23" t="inlineStr">
         <is>
           <t>No current cost</t>
         </is>
@@ -1727,9 +1727,9 @@
           <t>Stephen 9/22/26</t>
         </is>
       </c>
-      <c r="T14" s="19" t="inlineStr">
-        <is>
-          <t>Brand new payroll client.</t>
+      <c r="T14" s="20" t="inlineStr">
+        <is>
+          <t>Brand new payroll client, no current provider.</t>
         </is>
       </c>
     </row>
@@ -1749,7 +1749,7 @@
       </c>
       <c r="D15" s="1" t="inlineStr">
         <is>
-          <t>Existing</t>
+          <t>Existing (Gusto)</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
@@ -1797,11 +1797,11 @@
       </c>
       <c r="O15" s="4" t="n"/>
       <c r="P15" s="4" t="n"/>
-      <c r="Q15" s="5">
+      <c r="Q15" s="18">
         <f>M15+IF(ISNUMBER(O15),O15,0)+IF(ISNUMBER(P15),P15,0)</f>
         <v/>
       </c>
-      <c r="R15" s="21" t="inlineStr">
+      <c r="R15" s="22" t="inlineStr">
         <is>
           <t>Corrected</t>
         </is>
@@ -1811,9 +1811,9 @@
           <t>Stephen 9/22/26</t>
         </is>
       </c>
-      <c r="T15" s="19" t="inlineStr">
-        <is>
-          <t>Not on Paychex. On Gusto at $100/month, 2 employees, payroll only, no 401(k).</t>
+      <c r="T15" s="20" t="inlineStr">
+        <is>
+          <t>On Gusto at 100.00/month, 2 employees, payroll only, no 401(k). Not a Paychex client.</t>
         </is>
       </c>
     </row>
@@ -1833,7 +1833,7 @@
       </c>
       <c r="D16" s="1" t="inlineStr">
         <is>
-          <t>Existing</t>
+          <t>Existing (Gusto)</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
@@ -1881,11 +1881,11 @@
       </c>
       <c r="O16" s="4" t="n"/>
       <c r="P16" s="4" t="n"/>
-      <c r="Q16" s="5">
+      <c r="Q16" s="18">
         <f>M16+IF(ISNUMBER(O16),O16,0)+IF(ISNUMBER(P16),P16,0)</f>
         <v/>
       </c>
-      <c r="R16" s="21" t="inlineStr">
+      <c r="R16" s="22" t="inlineStr">
         <is>
           <t>Corrected</t>
         </is>
@@ -1895,9 +1895,9 @@
           <t>Stephen 9/22/26</t>
         </is>
       </c>
-      <c r="T16" s="19" t="inlineStr">
-        <is>
-          <t>On Gusto at $50/month, monthly. Sheet had $70.</t>
+      <c r="T16" s="20" t="inlineStr">
+        <is>
+          <t>On Gusto at 50.00/month, monthly. Original had 70.00.</t>
         </is>
       </c>
     </row>
@@ -1965,11 +1965,11 @@
       </c>
       <c r="O17" s="4" t="n"/>
       <c r="P17" s="4" t="n"/>
-      <c r="Q17" s="5">
+      <c r="Q17" s="18">
         <f>M17+IF(ISNUMBER(O17),O17,0)+IF(ISNUMBER(P17),P17,0)</f>
         <v/>
       </c>
-      <c r="R17" t="inlineStr">
+      <c r="R17" s="23" t="inlineStr">
         <is>
           <t>No current cost</t>
         </is>
@@ -1979,9 +1979,9 @@
           <t>Stephen 9/22/26</t>
         </is>
       </c>
-      <c r="T17" s="19" t="inlineStr">
-        <is>
-          <t>Brand new payroll client.</t>
+      <c r="T17" s="20" t="inlineStr">
+        <is>
+          <t>Brand new payroll client, no current provider.</t>
         </is>
       </c>
     </row>
@@ -2001,7 +2001,7 @@
       </c>
       <c r="D18" s="1" t="inlineStr">
         <is>
-          <t>Existing</t>
+          <t>Existing (IRS direct)</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
@@ -2049,11 +2049,11 @@
       </c>
       <c r="O18" s="4" t="n"/>
       <c r="P18" s="4" t="n"/>
-      <c r="Q18" s="5">
+      <c r="Q18" s="18">
         <f>M18+IF(ISNUMBER(O18),O18,0)+IF(ISNUMBER(P18),P18,0)</f>
         <v/>
       </c>
-      <c r="R18" s="21" t="inlineStr">
+      <c r="R18" s="22" t="inlineStr">
         <is>
           <t>Corrected</t>
         </is>
@@ -2063,9 +2063,9 @@
           <t>Stephen 9/22/26</t>
         </is>
       </c>
-      <c r="T18" s="19" t="inlineStr">
-        <is>
-          <t>No provider. Pays through IRS Treasury online, cash payroll, about $400/yr. Sheet had $300.</t>
+      <c r="T18" s="20" t="inlineStr">
+        <is>
+          <t>No provider. Pays through IRS Treasury online, cash payroll, about 400.00/yr. Original had 300.00.</t>
         </is>
       </c>
     </row>
@@ -2129,11 +2129,11 @@
       <c r="N19" s="6" t="n"/>
       <c r="O19" s="4" t="n"/>
       <c r="P19" s="4" t="n"/>
-      <c r="Q19" s="5">
+      <c r="Q19" s="18">
         <f>M19+IF(ISNUMBER(O19),O19,0)+IF(ISNUMBER(P19),P19,0)</f>
         <v/>
       </c>
-      <c r="R19" t="inlineStr">
+      <c r="R19" s="23" t="inlineStr">
         <is>
           <t>No current cost</t>
         </is>
@@ -2143,9 +2143,9 @@
           <t>—</t>
         </is>
       </c>
-      <c r="T19" s="19" t="inlineStr">
-        <is>
-          <t>Brand new payroll client.</t>
+      <c r="T19" s="20" t="inlineStr">
+        <is>
+          <t>Brand new payroll client, no current provider.</t>
         </is>
       </c>
     </row>
@@ -2213,11 +2213,11 @@
       </c>
       <c r="O20" s="4" t="n"/>
       <c r="P20" s="4" t="n"/>
-      <c r="Q20" s="5">
+      <c r="Q20" s="18">
         <f>M20+IF(ISNUMBER(O20),O20,0)+IF(ISNUMBER(P20),P20,0)</f>
         <v/>
       </c>
-      <c r="R20" t="inlineStr">
+      <c r="R20" s="23" t="inlineStr">
         <is>
           <t>No current cost</t>
         </is>
@@ -2227,9 +2227,9 @@
           <t>Stephen 9/22/26</t>
         </is>
       </c>
-      <c r="T20" s="19" t="inlineStr">
-        <is>
-          <t>Brand new payroll client.</t>
+      <c r="T20" s="20" t="inlineStr">
+        <is>
+          <t>Brand new payroll client, no current provider.</t>
         </is>
       </c>
     </row>
@@ -2415,7 +2415,7 @@
       <c r="I29" s="3" t="n"/>
       <c r="J29" s="3" t="n"/>
       <c r="K29" s="4" t="n"/>
-      <c r="L29" s="22" t="inlineStr">
+      <c r="L29" s="24" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
@@ -2427,7 +2427,7 @@
       <c r="N29" s="6" t="n"/>
       <c r="O29" s="4" t="n"/>
       <c r="P29" s="4" t="n"/>
-      <c r="Q29" s="23">
+      <c r="Q29" s="25">
         <f>SUM(Q3:Q26)</f>
         <v/>
       </c>
@@ -2446,7 +2446,7 @@
       <c r="I30" s="3" t="n"/>
       <c r="J30" s="3" t="n"/>
       <c r="K30" s="4" t="n"/>
-      <c r="L30" s="22" t="n"/>
+      <c r="L30" s="24" t="n"/>
       <c r="M30" s="11" t="n"/>
       <c r="N30" s="6" t="n"/>
       <c r="O30" s="4" t="n"/>
@@ -2467,7 +2467,7 @@
       <c r="I31" s="3" t="n"/>
       <c r="J31" s="3" t="n"/>
       <c r="K31" s="4" t="n"/>
-      <c r="L31" s="22" t="inlineStr">
+      <c r="L31" s="24" t="inlineStr">
         <is>
           <t>Multiplier</t>
         </is>
@@ -2479,7 +2479,10 @@
       <c r="N31" s="6" t="n"/>
       <c r="O31" s="4" t="n"/>
       <c r="P31" s="4" t="n"/>
-      <c r="Q31" s="5" t="n"/>
+      <c r="Q31" s="18">
+        <f>Q29*2</f>
+        <v/>
+      </c>
     </row>
     <row r="32" ht="15.75" customHeight="1" thickTop="1">
       <c r="A32" s="1" t="n">
@@ -2524,10 +2527,8 @@
       <c r="Q33" s="5" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="24" t="inlineStr">
-        <is>
-          <t>NOTES — updated 9/24/2026</t>
-        </is>
+      <c r="A34" s="1" t="n">
+        <v>32</v>
       </c>
       <c r="B34" s="1" t="n"/>
       <c r="C34" s="1" t="n"/>
@@ -2547,10 +2548,8 @@
       <c r="Q34" s="5" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="1" t="inlineStr">
-        <is>
-          <t>Pricing updated to what has been verified from actual Paychex invoices and retirement billing statements. Everything else on this sheet is unchanged from the original.</t>
-        </is>
+      <c r="A35" s="1" t="n">
+        <v>33</v>
       </c>
       <c r="B35" s="1" t="n"/>
       <c r="C35" s="1" t="n"/>
@@ -2570,7 +2569,9 @@
       <c r="Q35" s="5" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="1" t="inlineStr"/>
+      <c r="A36" s="1" t="n">
+        <v>34</v>
+      </c>
       <c r="B36" s="1" t="n"/>
       <c r="C36" s="1" t="n"/>
       <c r="D36" s="1" t="n"/>
@@ -2589,10 +2590,8 @@
       <c r="Q36" s="5" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="1" t="inlineStr">
-        <is>
-          <t>INCLUDED in Fee Per payroll run: every charge that hits each run. Delivery, Taxpay Locals, Direct Deposit Premium Processing, and the standing client discount.</t>
-        </is>
+      <c r="A37" s="1" t="n">
+        <v>35</v>
       </c>
       <c r="B37" s="1" t="n"/>
       <c r="C37" s="1" t="n"/>
@@ -2612,10 +2611,8 @@
       <c r="Q37" s="5" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="1" t="inlineStr">
-        <is>
-          <t>EXCLUDED: one-time setup fees, and Missing State ID / Missing Local ID penalties. Those stop once the registrations are filed.</t>
-        </is>
+      <c r="A38" s="1" t="n">
+        <v>36</v>
       </c>
       <c r="B38" s="1" t="n"/>
       <c r="C38" s="1" t="n"/>
@@ -2635,7 +2632,9 @@
       <c r="Q38" s="5" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="1" t="inlineStr"/>
+      <c r="A39" s="1" t="n">
+        <v>37</v>
+      </c>
       <c r="B39" s="1" t="n"/>
       <c r="C39" s="1" t="n"/>
       <c r="D39" s="1" t="n"/>
@@ -2654,10 +2653,8 @@
       <c r="Q39" s="5" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="1" t="inlineStr">
-        <is>
-          <t>401K Fees column is now the annual base (recordkeeping + 3(16) + participant fees). It does NOT include the setup fee installments.</t>
-        </is>
+      <c r="A40" s="1" t="n">
+        <v>38</v>
       </c>
       <c r="B40" s="1" t="n"/>
       <c r="C40" s="1" t="n"/>
@@ -2677,10 +2674,8 @@
       <c r="Q40" s="5" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="1" t="inlineStr">
-        <is>
-          <t>Outstanding 401(k) setup balances, separate from the annual figures above:</t>
-        </is>
+      <c r="A41" s="1" t="n">
+        <v>39</v>
       </c>
       <c r="B41" s="1" t="n"/>
       <c r="C41" s="1" t="n"/>
@@ -2700,10 +2695,8 @@
       <c r="Q41" s="5" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     Walters Mirrors     2,749.07     of 2,999.00</t>
-        </is>
+      <c r="A42" s="1" t="n">
+        <v>40</v>
       </c>
       <c r="B42" s="1" t="n"/>
       <c r="C42" s="1" t="n"/>
@@ -2723,10 +2716,8 @@
       <c r="Q42" s="5" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     Onchain Strategies  3,887.91     of 3,999.00</t>
-        </is>
+      <c r="A43" s="1" t="n">
+        <v>41</v>
       </c>
       <c r="B43" s="1" t="n"/>
       <c r="C43" s="1" t="n"/>
@@ -2746,10 +2737,8 @@
       <c r="Q43" s="5" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     Spencer Thwaytes    3,999.00     of 3,999.00, nothing collected yet</t>
-        </is>
+      <c r="A44" s="1" t="n">
+        <v>42</v>
       </c>
       <c r="B44" s="1" t="n"/>
       <c r="C44" s="1" t="n"/>
@@ -2769,10 +2758,8 @@
       <c r="Q44" s="5" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="1" t="inlineStr">
-        <is>
-          <t xml:space="preserve">     Each plan also carries a 1,500 transfer fee on exit.</t>
-        </is>
+      <c r="A45" s="1" t="n">
+        <v>43</v>
       </c>
       <c r="B45" s="1" t="n"/>
       <c r="C45" s="1" t="n"/>
@@ -2792,7 +2779,9 @@
       <c r="Q45" s="5" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="1" t="inlineStr"/>
+      <c r="A46" s="1" t="n">
+        <v>44</v>
+      </c>
       <c r="B46" s="1" t="n"/>
       <c r="C46" s="1" t="n"/>
       <c r="D46" s="1" t="n"/>
@@ -2811,10 +2800,8 @@
       <c r="Q46" s="5" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="1" t="inlineStr">
-        <is>
-          <t>STILL NO INVOICE: Upstate Logistics, Tyree Advisory, Kranz Motorcars, RJC Holdings. Those four rows are still the original figures.</t>
-        </is>
+      <c r="A47" s="1" t="n">
+        <v>45</v>
       </c>
       <c r="B47" s="1" t="n"/>
       <c r="C47" s="1" t="n"/>
@@ -2834,7 +2821,9 @@
       <c r="Q47" s="5" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="1" t="inlineStr"/>
+      <c r="A48" s="1" t="n">
+        <v>46</v>
+      </c>
       <c r="B48" s="1" t="n"/>
       <c r="C48" s="1" t="n"/>
       <c r="D48" s="1" t="n"/>
@@ -2853,10 +2842,8 @@
       <c r="Q48" s="5" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="1" t="inlineStr">
-        <is>
-          <t>The Multiplier row applies 2x to every client including the new ones. Grid pays 2x on annualized ADP revenue for Paychex conversions only, so that row is not a payout figure.</t>
-        </is>
+      <c r="A49" s="1" t="n">
+        <v>47</v>
       </c>
       <c r="B49" s="1" t="n"/>
       <c r="C49" s="1" t="n"/>
@@ -4447,4 +4434,207 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" horizontalDpi="4294967293" verticalDpi="0"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="125" customWidth="1" min="1" max="1"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="15" t="inlineStr">
+        <is>
+          <t>WHAT CHANGED ON THIS SHEET — 9/24/2026</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>Pricing is now what has been verified from actual Paychex invoices and retirement billing statements.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>Columns R, S and T were added: whether a row is verified, the source, and a note. Nothing else was removed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr"/>
+    </row>
+    <row r="6">
+      <c r="A6" s="15" t="inlineStr">
+        <is>
+          <t>CELLS CHANGED, besides Fee Per payroll run:</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Walters Mirrors — employees 5 to 3, frequency Semi Monthly to Biweekly, runs 24 to 26. The invoice shows 3 active employees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Upstate Logistics — 401(k) fees 0.91 to 0. That charge was not a plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Complete Merchant, FRG, Broadway 2000 — status now reads Existing, with the provider named.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   401(k) fees for Onchain, Walters and Spencer Thwaytes replaced with the verified annual base.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Column Q, Total Current Annualized Billings, was empty and is now run rate plus 401(k) plus other fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="15" t="inlineStr">
+        <is>
+          <t>WHAT IS IN THE FEE PER PAYROLL RUN</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Every charge that hits each run: Delivery, Taxpay Locals, Direct Deposit Premium Processing, and the standing client discount.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Excluded: one-time setup fees, and Missing State ID or Missing Local ID penalties, which stop once the registrations are filed.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>401(K) FEES COLUMN</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   This is the annual recurring base only: recordkeeping, 3(16) administration, and per-participant fees.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   It does not include the setup fee installments, which are separate and one-time.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Outstanding setup balances, from the Paychex retirement billing statements:</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Walters Mirrors        2,749.07 remaining of 2,999.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Onchain Strategies     3,887.91 remaining of 3,999.00</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Spencer Thwaytes       3,999.00 remaining of 3,999.00, nothing collected yet</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr"/>
+    </row>
+    <row r="25">
+      <c r="A25" s="15" t="inlineStr">
+        <is>
+          <t>STILL NO INVOICE</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Upstate Logistics, Tyree Advisory, Kranz Motorcars, RJC Holdings. Those four rows are still the original figures.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr"/>
+    </row>
+    <row r="28">
+      <c r="A28" s="15" t="inlineStr">
+        <is>
+          <t>ON THE MULTIPLIER ROW</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   That row applies 2x to every client on the sheet. This sheet holds current-provider pricing across Paychex, Gusto,</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   IRS-direct and brand-new clients, and none of it is an ADP price. It is not a payout figure.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
CBA: add 401(k) comp (750 conversion / 300 new) and mark new clients one-time payment
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HvXhTSq2hCmheT3mKtqmHP
</commit_message>
<xml_diff>
--- a/output/stephen/CBA_Innovative_Advisors_Updated_2026-09-24.xlsx
+++ b/output/stephen/CBA_Innovative_Advisors_Updated_2026-09-24.xlsx
@@ -16,10 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="165" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
+    <numFmt numFmtId="167" formatCode="$#,##0"/>
   </numFmts>
   <fonts count="8">
     <font>
@@ -74,7 +75,7 @@
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="7">
+  <fills count="8">
     <fill>
       <patternFill/>
     </fill>
@@ -105,6 +106,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00D9D9D9"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
   </fills>
@@ -165,7 +171,7 @@
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -248,6 +254,9 @@
     <xf numFmtId="166" fontId="7" fillId="0" borderId="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="1">
       <protection locked="0" hidden="0"/>
     </xf>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -593,7 +602,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A2:T122"/>
+  <dimension ref="A2:V122"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="15.5703125" defaultRowHeight="15"/>
   <cols>
     <col width="14.28515625" bestFit="1" customWidth="1" min="1" max="1"/>
@@ -609,6 +618,8 @@
     <col width="14" customWidth="1" min="18" max="18"/>
     <col width="32" customWidth="1" min="19" max="19"/>
     <col width="88" customWidth="1" min="20" max="20"/>
+    <col width="14" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="2" ht="74.45" customHeight="1">
@@ -712,6 +723,16 @@
           <t>Notes</t>
         </is>
       </c>
+      <c r="U2" s="15" t="inlineStr">
+        <is>
+          <t>401(k) Comp</t>
+        </is>
+      </c>
+      <c r="V2" s="15" t="inlineStr">
+        <is>
+          <t>Payroll Comp</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="1" t="n">
@@ -1136,6 +1157,9 @@
           <t>Base is Officer Only Payroll 65.00, not 58.00, plus Delivery 36.00. 401(k) recurring 181.00/mo = 2,172.00/yr.</t>
         </is>
       </c>
+      <c r="U7" s="26" t="n">
+        <v>750</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="1" t="n">
@@ -1392,6 +1416,9 @@
           <t>HR Pro is a bundled HR and payroll fee, 896.70 less 394.55 discount = 502.15 per run, bi-weekly. Invoice shows 3 active employees, not 5. 401(k) recurring 193.00/mo = 2,316.00/yr.</t>
         </is>
       </c>
+      <c r="U10" s="26" t="n">
+        <v>750</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="n">
@@ -1479,6 +1506,9 @@
         <is>
           <t>Express Payroll 77.00 matches the original. 401(k) recurring 175.00/mo = 2,100.00/yr.</t>
         </is>
+      </c>
+      <c r="U11" s="26" t="n">
+        <v>750</v>
       </c>
     </row>
     <row r="12">
@@ -1648,6 +1678,9 @@
           <t>Set up at Paychex but has never run a payroll, so there is no current billing.</t>
         </is>
       </c>
+      <c r="U13" s="26" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="n">
@@ -1732,6 +1765,14 @@
           <t>Brand new payroll client, no current provider.</t>
         </is>
       </c>
+      <c r="U14" s="26" t="n">
+        <v>300</v>
+      </c>
+      <c r="V14" s="27" t="inlineStr">
+        <is>
+          <t>One-time payment</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="n">
@@ -1816,6 +1857,9 @@
           <t>On Gusto at 100.00/month, 2 employees, payroll only, no 401(k). Not a Paychex client.</t>
         </is>
       </c>
+      <c r="U15" s="26" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
@@ -1900,6 +1944,9 @@
           <t>On Gusto at 50.00/month, monthly. Original had 70.00.</t>
         </is>
       </c>
+      <c r="U16" s="26" t="n">
+        <v>300</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
@@ -1984,6 +2031,14 @@
           <t>Brand new payroll client, no current provider.</t>
         </is>
       </c>
+      <c r="U17" s="26" t="n">
+        <v>300</v>
+      </c>
+      <c r="V17" s="27" t="inlineStr">
+        <is>
+          <t>One-time payment</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
@@ -2067,6 +2122,9 @@
         <is>
           <t>No provider. Pays through IRS Treasury online, cash payroll, about 400.00/yr. Original had 300.00.</t>
         </is>
+      </c>
+      <c r="U18" s="26" t="n">
+        <v>300</v>
       </c>
     </row>
     <row r="19">
@@ -2148,6 +2206,11 @@
           <t>Brand new payroll client, no current provider.</t>
         </is>
       </c>
+      <c r="V19" s="27" t="inlineStr">
+        <is>
+          <t>One-time payment</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
@@ -2230,6 +2293,14 @@
       <c r="T20" s="20" t="inlineStr">
         <is>
           <t>Brand new payroll client, no current provider.</t>
+        </is>
+      </c>
+      <c r="U20" s="26" t="n">
+        <v>300</v>
+      </c>
+      <c r="V20" s="27" t="inlineStr">
+        <is>
+          <t>One-time payment</t>
         </is>
       </c>
     </row>
@@ -2429,6 +2500,10 @@
       <c r="P29" s="4" t="n"/>
       <c r="Q29" s="25">
         <f>SUM(Q3:Q26)</f>
+        <v/>
+      </c>
+      <c r="U29" s="28">
+        <f>SUM(U3:U26)</f>
         <v/>
       </c>
     </row>
@@ -4442,7 +4517,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A30"/>
+  <dimension ref="A1:A37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="125" customWidth="1" min="1" max="1"/>
@@ -4455,9 +4530,6 @@
         </is>
       </c>
     </row>
-    <row r="2">
-      <c r="A2" t="inlineStr"/>
-    </row>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -4472,9 +4544,6 @@
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" t="inlineStr"/>
-    </row>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
@@ -4517,9 +4586,6 @@
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" t="inlineStr"/>
-    </row>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
@@ -4541,9 +4607,6 @@
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" t="inlineStr"/>
-    </row>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
@@ -4593,9 +4656,6 @@
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" t="inlineStr"/>
-    </row>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
@@ -4610,9 +4670,6 @@
         </is>
       </c>
     </row>
-    <row r="27">
-      <c r="A27" t="inlineStr"/>
-    </row>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
@@ -4631,6 +4688,48 @@
       <c r="A30" t="inlineStr">
         <is>
           <t xml:space="preserve">   IRS-direct and brand-new clients, and none of it is an ADP price. It is not a payout figure.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="15" t="inlineStr">
+        <is>
+          <t>401(K) COMP AND PAYROLL COMP — columns U and V</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   401(k) comp is 750 per Paychex conversion and 300 per new plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Conversions, 750 each: Onchain Strategies, Walters Mirrors, Spencer Thwaytes.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        New plans, 300 each: B333, AJG, Complete Merchant, FRG, Kapstone, Broadway 2000, North Star.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t xml:space="preserve">        Total 4,350.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Payroll comp column marks the new clients as a one-time payment rather than the 2x conversion multiple.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
CBA: 401k new comp to 350, verification by invoice or email, separate Platinum tab for new clients
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HvXhTSq2hCmheT3mKtqmHP
</commit_message>
<xml_diff>
--- a/output/stephen/CBA_Innovative_Advisors_Updated_2026-09-24.xlsx
+++ b/output/stephen/CBA_Innovative_Advisors_Updated_2026-09-24.xlsx
@@ -7,7 +7,8 @@
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Notes 9-24-26" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="New Clients - Platinum" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Notes 9-24-26" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="191029" fullCalcOnLoad="1"/>
@@ -22,7 +23,7 @@
     <numFmt numFmtId="166" formatCode="$#,##0.00"/>
     <numFmt numFmtId="167" formatCode="$#,##0"/>
   </numFmts>
-  <fonts count="8">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -74,8 +75,22 @@
     <font>
       <b val="1"/>
     </font>
+    <font/>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="14"/>
+    </font>
+    <font>
+      <i val="1"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
   </fonts>
-  <fills count="8">
+  <fills count="10">
     <fill>
       <patternFill/>
     </fill>
@@ -113,8 +128,18 @@
         <fgColor rgb="00FFF2CC"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEBF7"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C00000"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="4">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -165,13 +190,27 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="00BFBFBF"/>
+      </left>
+      <right style="thin">
+        <color rgb="00BFBFBF"/>
+      </right>
+      <top style="thin">
+        <color rgb="00BFBFBF"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00BFBFBF"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="45">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -257,6 +296,24 @@
     <xf numFmtId="167" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="167" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="8" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="7" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="6" borderId="4" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="7" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="7" fillId="7" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="7" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -615,7 +672,7 @@
     <col width="15" customWidth="1" min="12" max="12"/>
     <col width="15" customWidth="1" min="15" max="16"/>
     <col width="18" bestFit="1" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
+    <col width="24" customWidth="1" min="18" max="18"/>
     <col width="32" customWidth="1" min="19" max="19"/>
     <col width="88" customWidth="1" min="20" max="20"/>
     <col width="14" customWidth="1" min="21" max="21"/>
@@ -802,9 +859,9 @@
         <f>M3+IF(ISNUMBER(O3),O3,0)+IF(ISNUMBER(P3),P3,0)</f>
         <v/>
       </c>
-      <c r="R3" s="19" t="inlineStr">
-        <is>
-          <t>Verified</t>
+      <c r="R3" s="29" t="inlineStr">
+        <is>
+          <t>Verified - invoice</t>
         </is>
       </c>
       <c r="S3" t="inlineStr">
@@ -886,9 +943,9 @@
         <f>M4+IF(ISNUMBER(O4),O4,0)+IF(ISNUMBER(P4),P4,0)</f>
         <v/>
       </c>
-      <c r="R4" s="21" t="inlineStr">
-        <is>
-          <t>Not verified</t>
+      <c r="R4" s="30" t="inlineStr">
+        <is>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="S4" t="inlineStr">
@@ -970,9 +1027,9 @@
         <f>M5+IF(ISNUMBER(O5),O5,0)+IF(ISNUMBER(P5),P5,0)</f>
         <v/>
       </c>
-      <c r="R5" s="22" t="inlineStr">
-        <is>
-          <t>Corrected</t>
+      <c r="R5" s="29" t="inlineStr">
+        <is>
+          <t>Verified - invoice</t>
         </is>
       </c>
       <c r="S5" t="inlineStr">
@@ -1054,9 +1111,9 @@
         <f>M6+IF(ISNUMBER(O6),O6,0)+IF(ISNUMBER(P6),P6,0)</f>
         <v/>
       </c>
-      <c r="R6" s="21" t="inlineStr">
-        <is>
-          <t>Not verified</t>
+      <c r="R6" s="30" t="inlineStr">
+        <is>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="S6" t="inlineStr">
@@ -1142,9 +1199,9 @@
         <f>M7+IF(ISNUMBER(O7),O7,0)+IF(ISNUMBER(P7),P7,0)</f>
         <v/>
       </c>
-      <c r="R7" s="22" t="inlineStr">
-        <is>
-          <t>Corrected</t>
+      <c r="R7" s="29" t="inlineStr">
+        <is>
+          <t>Verified - invoice</t>
         </is>
       </c>
       <c r="S7" t="inlineStr">
@@ -1229,9 +1286,9 @@
         <f>M8+IF(ISNUMBER(O8),O8,0)+IF(ISNUMBER(P8),P8,0)</f>
         <v/>
       </c>
-      <c r="R8" s="21" t="inlineStr">
-        <is>
-          <t>Not verified</t>
+      <c r="R8" s="30" t="inlineStr">
+        <is>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="S8" t="inlineStr">
@@ -1313,9 +1370,9 @@
         <f>M9+IF(ISNUMBER(O9),O9,0)+IF(ISNUMBER(P9),P9,0)</f>
         <v/>
       </c>
-      <c r="R9" s="19" t="inlineStr">
-        <is>
-          <t>Verified</t>
+      <c r="R9" s="29" t="inlineStr">
+        <is>
+          <t>Verified - invoice</t>
         </is>
       </c>
       <c r="S9" t="inlineStr">
@@ -1401,9 +1458,9 @@
         <f>M10+IF(ISNUMBER(O10),O10,0)+IF(ISNUMBER(P10),P10,0)</f>
         <v/>
       </c>
-      <c r="R10" s="22" t="inlineStr">
-        <is>
-          <t>Corrected</t>
+      <c r="R10" s="29" t="inlineStr">
+        <is>
+          <t>Verified - invoice</t>
         </is>
       </c>
       <c r="S10" t="inlineStr">
@@ -1492,9 +1549,9 @@
         <f>M11+IF(ISNUMBER(O11),O11,0)+IF(ISNUMBER(P11),P11,0)</f>
         <v/>
       </c>
-      <c r="R11" s="19" t="inlineStr">
-        <is>
-          <t>Verified</t>
+      <c r="R11" s="29" t="inlineStr">
+        <is>
+          <t>Verified - invoice</t>
         </is>
       </c>
       <c r="S11" t="inlineStr">
@@ -1579,9 +1636,9 @@
         <f>M12+IF(ISNUMBER(O12),O12,0)+IF(ISNUMBER(P12),P12,0)</f>
         <v/>
       </c>
-      <c r="R12" s="21" t="inlineStr">
-        <is>
-          <t>Not verified</t>
+      <c r="R12" s="30" t="inlineStr">
+        <is>
+          <t>MISSING</t>
         </is>
       </c>
       <c r="S12" t="inlineStr">
@@ -1663,9 +1720,9 @@
         <f>M13+IF(ISNUMBER(O13),O13,0)+IF(ISNUMBER(P13),P13,0)</f>
         <v/>
       </c>
-      <c r="R13" s="23" t="inlineStr">
-        <is>
-          <t>No current cost</t>
+      <c r="R13" s="31" t="inlineStr">
+        <is>
+          <t>Verified - Stephen's email</t>
         </is>
       </c>
       <c r="S13" t="inlineStr">
@@ -1679,7 +1736,7 @@
         </is>
       </c>
       <c r="U13" s="26" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
     </row>
     <row r="14">
@@ -1750,9 +1807,9 @@
         <f>M14+IF(ISNUMBER(O14),O14,0)+IF(ISNUMBER(P14),P14,0)</f>
         <v/>
       </c>
-      <c r="R14" s="23" t="inlineStr">
-        <is>
-          <t>No current cost</t>
+      <c r="R14" s="32" t="inlineStr">
+        <is>
+          <t>New client</t>
         </is>
       </c>
       <c r="S14" t="inlineStr">
@@ -1766,7 +1823,7 @@
         </is>
       </c>
       <c r="U14" s="26" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="V14" s="27" t="inlineStr">
         <is>
@@ -1842,9 +1899,9 @@
         <f>M15+IF(ISNUMBER(O15),O15,0)+IF(ISNUMBER(P15),P15,0)</f>
         <v/>
       </c>
-      <c r="R15" s="22" t="inlineStr">
-        <is>
-          <t>Corrected</t>
+      <c r="R15" s="31" t="inlineStr">
+        <is>
+          <t>Verified - Stephen's email</t>
         </is>
       </c>
       <c r="S15" t="inlineStr">
@@ -1858,7 +1915,7 @@
         </is>
       </c>
       <c r="U15" s="26" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
     </row>
     <row r="16">
@@ -1929,9 +1986,9 @@
         <f>M16+IF(ISNUMBER(O16),O16,0)+IF(ISNUMBER(P16),P16,0)</f>
         <v/>
       </c>
-      <c r="R16" s="22" t="inlineStr">
-        <is>
-          <t>Corrected</t>
+      <c r="R16" s="31" t="inlineStr">
+        <is>
+          <t>Verified - Stephen's email</t>
         </is>
       </c>
       <c r="S16" t="inlineStr">
@@ -1945,7 +2002,7 @@
         </is>
       </c>
       <c r="U16" s="26" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
     </row>
     <row r="17">
@@ -2016,9 +2073,9 @@
         <f>M17+IF(ISNUMBER(O17),O17,0)+IF(ISNUMBER(P17),P17,0)</f>
         <v/>
       </c>
-      <c r="R17" s="23" t="inlineStr">
-        <is>
-          <t>No current cost</t>
+      <c r="R17" s="32" t="inlineStr">
+        <is>
+          <t>New client</t>
         </is>
       </c>
       <c r="S17" t="inlineStr">
@@ -2032,7 +2089,7 @@
         </is>
       </c>
       <c r="U17" s="26" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="V17" s="27" t="inlineStr">
         <is>
@@ -2108,9 +2165,9 @@
         <f>M18+IF(ISNUMBER(O18),O18,0)+IF(ISNUMBER(P18),P18,0)</f>
         <v/>
       </c>
-      <c r="R18" s="22" t="inlineStr">
-        <is>
-          <t>Corrected</t>
+      <c r="R18" s="31" t="inlineStr">
+        <is>
+          <t>Verified - Stephen's email</t>
         </is>
       </c>
       <c r="S18" t="inlineStr">
@@ -2124,7 +2181,7 @@
         </is>
       </c>
       <c r="U18" s="26" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
     </row>
     <row r="19">
@@ -2191,9 +2248,9 @@
         <f>M19+IF(ISNUMBER(O19),O19,0)+IF(ISNUMBER(P19),P19,0)</f>
         <v/>
       </c>
-      <c r="R19" s="23" t="inlineStr">
-        <is>
-          <t>No current cost</t>
+      <c r="R19" s="32" t="inlineStr">
+        <is>
+          <t>New client</t>
         </is>
       </c>
       <c r="S19" t="inlineStr">
@@ -2280,9 +2337,9 @@
         <f>M20+IF(ISNUMBER(O20),O20,0)+IF(ISNUMBER(P20),P20,0)</f>
         <v/>
       </c>
-      <c r="R20" s="23" t="inlineStr">
-        <is>
-          <t>No current cost</t>
+      <c r="R20" s="32" t="inlineStr">
+        <is>
+          <t>New client</t>
         </is>
       </c>
       <c r="S20" t="inlineStr">
@@ -2296,7 +2353,7 @@
         </is>
       </c>
       <c r="U20" s="26" t="n">
-        <v>300</v>
+        <v>350</v>
       </c>
       <c r="V20" s="27" t="inlineStr">
         <is>
@@ -4517,7 +4574,355 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A37"/>
+  <dimension ref="A1:J17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="22" customWidth="1" min="1" max="1"/>
+    <col width="34" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="14" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="26" customHeight="1">
+      <c r="A1" s="33" t="inlineStr">
+        <is>
+          <t>NEW CLIENTS — PLATINUM, NOT GRID</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="34" t="inlineStr">
+        <is>
+          <t>These are brand new payroll clients with no current provider. They are not part of the Grid submission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="32" customHeight="1">
+      <c r="A4" s="35" t="inlineStr">
+        <is>
+          <t>Owner</t>
+        </is>
+      </c>
+      <c r="B4" s="35" t="inlineStr">
+        <is>
+          <t>Client Legal Name</t>
+        </is>
+      </c>
+      <c r="C4" s="35" t="inlineStr">
+        <is>
+          <t>EIN</t>
+        </is>
+      </c>
+      <c r="D4" s="35" t="inlineStr">
+        <is>
+          <t>EE</t>
+        </is>
+      </c>
+      <c r="E4" s="35" t="inlineStr">
+        <is>
+          <t>Frequency</t>
+        </is>
+      </c>
+      <c r="F4" s="35" t="inlineStr">
+        <is>
+          <t>Runs/yr</t>
+        </is>
+      </c>
+      <c r="G4" s="35" t="inlineStr">
+        <is>
+          <t>Proposed ADP fee per run</t>
+        </is>
+      </c>
+      <c r="H4" s="35" t="inlineStr">
+        <is>
+          <t>Annual ADP revenue</t>
+        </is>
+      </c>
+      <c r="I4" s="35" t="inlineStr">
+        <is>
+          <t>401(k) plan</t>
+        </is>
+      </c>
+      <c r="J4" s="35" t="inlineStr">
+        <is>
+          <t>401(k) comp</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="36" t="inlineStr">
+        <is>
+          <t>Anthony Gerb</t>
+        </is>
+      </c>
+      <c r="B5" s="36" t="inlineStr">
+        <is>
+          <t>AJG Trading LLC</t>
+        </is>
+      </c>
+      <c r="C5" s="36" t="inlineStr">
+        <is>
+          <t>41-5035542</t>
+        </is>
+      </c>
+      <c r="D5" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E5" s="36" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F5" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="G5" s="37" t="n">
+        <v>70</v>
+      </c>
+      <c r="H5" s="37">
+        <f>F5*G5</f>
+        <v/>
+      </c>
+      <c r="I5" s="36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J5" s="38" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="36" t="inlineStr">
+        <is>
+          <t>Alexander Harris</t>
+        </is>
+      </c>
+      <c r="B6" s="36" t="inlineStr">
+        <is>
+          <t>Kapstone Digital LLC</t>
+        </is>
+      </c>
+      <c r="C6" s="36" t="inlineStr">
+        <is>
+          <t>85-3782692</t>
+        </is>
+      </c>
+      <c r="D6" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E6" s="36" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F6" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="G6" s="37" t="n">
+        <v>70</v>
+      </c>
+      <c r="H6" s="37">
+        <f>F6*G6</f>
+        <v/>
+      </c>
+      <c r="I6" s="36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J6" s="38" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="36" t="inlineStr">
+        <is>
+          <t>John Ewing</t>
+        </is>
+      </c>
+      <c r="B7" s="36" t="inlineStr">
+        <is>
+          <t>Atlas Opera, Inc.</t>
+        </is>
+      </c>
+      <c r="C7" s="36" t="inlineStr">
+        <is>
+          <t>82-2302400</t>
+        </is>
+      </c>
+      <c r="D7" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E7" s="36" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F7" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="G7" s="37" t="n">
+        <v>70</v>
+      </c>
+      <c r="H7" s="37">
+        <f>F7*G7</f>
+        <v/>
+      </c>
+      <c r="I7" s="36" t="inlineStr"/>
+      <c r="J7" s="36" t="n"/>
+    </row>
+    <row r="8">
+      <c r="A8" s="36" t="inlineStr">
+        <is>
+          <t>Christina Pellicane</t>
+        </is>
+      </c>
+      <c r="B8" s="36" t="inlineStr">
+        <is>
+          <t>North Star Works, LLC</t>
+        </is>
+      </c>
+      <c r="C8" s="36" t="inlineStr">
+        <is>
+          <t>42-4495054</t>
+        </is>
+      </c>
+      <c r="D8" s="36" t="n">
+        <v>1</v>
+      </c>
+      <c r="E8" s="36" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F8" s="36" t="n">
+        <v>12</v>
+      </c>
+      <c r="G8" s="37" t="n">
+        <v>50</v>
+      </c>
+      <c r="H8" s="37">
+        <f>F8*G8</f>
+        <v/>
+      </c>
+      <c r="I8" s="36" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="J8" s="38" t="n">
+        <v>350</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="39" t="n"/>
+      <c r="B9" s="39" t="inlineStr">
+        <is>
+          <t>TOTAL</t>
+        </is>
+      </c>
+      <c r="C9" s="39" t="n"/>
+      <c r="D9" s="39" t="n"/>
+      <c r="E9" s="39" t="n"/>
+      <c r="F9" s="39" t="n"/>
+      <c r="G9" s="39" t="n"/>
+      <c r="H9" s="40">
+        <f>SUM(H5:H8)</f>
+        <v/>
+      </c>
+      <c r="I9" s="39" t="n"/>
+      <c r="J9" s="41">
+        <f>SUM(J5:J8)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="42" t="inlineStr">
+        <is>
+          <t>PAYOUT</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>Platinum, 1x annualized ADP revenue</t>
+        </is>
+      </c>
+      <c r="C12" s="43">
+        <f>H9</f>
+        <v/>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Applies to the four clients above.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>401(k) comp, 350 per new plan</t>
+        </is>
+      </c>
+      <c r="C13" s="43">
+        <f>J9</f>
+        <v/>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Three of the four have a plan.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="15" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="C14" s="44">
+        <f>C12+C13</f>
+        <v/>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>Proposed ADP pricing is carried over from the original sheet. These clients have no current provider, so there is nothing to compare against.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Platinum pays 1x. The Grid 2x multiple on the main tab applies to Paychex conversions only.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:A46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="125" customWidth="1" min="1" max="1"/>
@@ -4530,6 +4935,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
@@ -4544,6 +4950,7 @@
         </is>
       </c>
     </row>
+    <row r="5"/>
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
@@ -4586,6 +4993,7 @@
         </is>
       </c>
     </row>
+    <row r="12"/>
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
@@ -4607,6 +5015,7 @@
         </is>
       </c>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
@@ -4656,6 +5065,7 @@
         </is>
       </c>
     </row>
+    <row r="24"/>
     <row r="25">
       <c r="A25" s="15" t="inlineStr">
         <is>
@@ -4670,6 +5080,7 @@
         </is>
       </c>
     </row>
+    <row r="27"/>
     <row r="28">
       <c r="A28" s="15" t="inlineStr">
         <is>
@@ -4691,6 +5102,7 @@
         </is>
       </c>
     </row>
+    <row r="31"/>
     <row r="32">
       <c r="A32" s="15" t="inlineStr">
         <is>
@@ -4699,37 +5111,92 @@
       </c>
     </row>
     <row r="33">
-      <c r="A33" t="inlineStr">
-        <is>
-          <t xml:space="preserve">   401(k) comp is 750 per Paychex conversion and 300 per new plan.</t>
+      <c r="A33" s="15" t="inlineStr">
+        <is>
+          <t>VERIFICATION — column R</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Conversions, 750 each: Onchain Strategies, Walters Mirrors, Spencer Thwaytes.</t>
+          <t xml:space="preserve">   Verified - invoice (6): Wisdom by Woods, Auction Time Pieces, Backfin, Walters Mirrors, Onchain, Spencer Thwaytes.</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t xml:space="preserve">        New plans, 300 each: B333, AJG, Complete Merchant, FRG, Kapstone, Broadway 2000, North Star.</t>
+          <t xml:space="preserve">   Verified - Stephen's email (4): B333, Complete Merchant, FRG Advisory, Broadway 2000.</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t xml:space="preserve">        Total 4,350.</t>
+          <t xml:space="preserve">   MISSING (4): Upstate Logistics, Tyree Advisory, Kranz Motorcars, RJC Holdings. Still on the original figures.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t xml:space="preserve">   Payroll comp column marks the new clients as a one-time payment rather than the 2x conversion multiple.</t>
+          <t xml:space="preserve">   New client (4): AJG, Kapstone, Atlas Opera, North Star. See the Platinum tab.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr"/>
+    </row>
+    <row r="39">
+      <c r="A39" s="15" t="inlineStr">
+        <is>
+          <t>401(K) COMP — column U</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   750 per Paychex conversion: Onchain, Walters Mirrors, Spencer Thwaytes. 2,250 total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   350 per new plan: B333, AJG, Complete Merchant, FRG, Kapstone, Broadway 2000, North Star. 2,450 total.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   401(k) comp overall: 4,700.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr"/>
+    </row>
+    <row r="44">
+      <c r="A44" s="15" t="inlineStr">
+        <is>
+          <t>NEW CLIENTS — separate tab</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   AJG, Kapstone, Atlas Opera and North Star are on their own tab. They are Platinum at 1x, not part of the Grid submission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">   Their payout is calculated there and kept out of the main total.</t>
         </is>
       </c>
     </row>

</xml_diff>